<commit_message>
Use Hebrew geresh in flashcard loanwords
</commit_message>
<xml_diff>
--- a/etc/hebrew/nouns.xlsx
+++ b/etc/hebrew/nouns.xlsx
@@ -3323,18 +3323,18 @@
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>גִּ'ירָף</t>
+          <t>גִּ׳ירָף</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>גִּ'ירָפָה</t>
+          <t>גִּ׳ירָפָה</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr"/>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>גִּ'ירָפוֹת</t>
+          <t>גִּ׳ירָפוֹת</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr"/>

</xml_diff>